<commit_message>
Update PBPK workflows, simulations, and manuscript
</commit_message>
<xml_diff>
--- a/00_Data/Human/Parameters_human.xlsx
+++ b/00_Data/Human/Parameters_human.xlsx
@@ -1,31 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\KrinaMehta\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABA1EDF9-AB5F-43EA-A1B1-0530BFB8D00B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Included" sheetId="1" r:id="rId1"/>
+    <sheet name="Included" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0" iterateDelta="1E-4"/>
-  <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="72">
   <si>
     <t>Drug Name</t>
   </si>
@@ -238,19 +226,28 @@
   </si>
   <si>
     <t>Benamara et al., 2026; PMID: 41536283</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1/min</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -273,17 +270,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="11" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -476,20 +469,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G49"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="23.1796875" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="32" customWidth="1"/>
-    <col min="4" max="4" width="18.54296875" customWidth="1"/>
-    <col min="5" max="5" width="10.26953125" customWidth="1"/>
-    <col min="6" max="6" width="42" customWidth="1"/>
-    <col min="7" max="7" width="60" customWidth="1"/>
+    <col min="1" max="1" width="23.1796875" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="32" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="18.54296875" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="10.26953125" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="42" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="60" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -512,7 +505,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -522,7 +515,7 @@
       <c r="C2" t="s">
         <v>9</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="n">
         <v>0.65</v>
       </c>
       <c r="E2" t="s">
@@ -535,7 +528,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" ht="28.5" customHeight="1">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -545,8 +538,8 @@
       <c r="C3" t="s">
         <v>13</v>
       </c>
-      <c r="D3">
-        <v>0.29899999999999999</v>
+      <c r="D3" t="n">
+        <v>0.000299</v>
       </c>
       <c r="E3" t="s">
         <v>10</v>
@@ -558,7 +551,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -568,7 +561,7 @@
       <c r="C4" t="s">
         <v>15</v>
       </c>
-      <c r="D4">
+      <c r="D4" t="n">
         <v>9.3600000000000003E-3</v>
       </c>
       <c r="E4" t="s">
@@ -581,7 +574,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" ht="28.5" customHeight="1">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -591,7 +584,7 @@
       <c r="C5" t="s">
         <v>17</v>
       </c>
-      <c r="D5">
+      <c r="D5" t="n">
         <v>0.60599999999999998</v>
       </c>
       <c r="E5" t="s">
@@ -604,7 +597,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -614,7 +607,7 @@
       <c r="C6" t="s">
         <v>20</v>
       </c>
-      <c r="D6">
+      <c r="D6" t="n">
         <v>0.60899999999999999</v>
       </c>
       <c r="E6" t="s">
@@ -627,7 +620,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -637,7 +630,7 @@
       <c r="C7" t="s">
         <v>23</v>
       </c>
-      <c r="D7">
+      <c r="D7" t="n">
         <v>4.2599999999999999E-2</v>
       </c>
       <c r="E7" t="s">
@@ -650,7 +643,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -660,7 +653,7 @@
       <c r="C8" t="s">
         <v>9</v>
       </c>
-      <c r="D8">
+      <c r="D8" t="n">
         <v>1.07</v>
       </c>
       <c r="E8" t="s">
@@ -673,7 +666,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9">
       <c r="A9" t="s">
         <v>25</v>
       </c>
@@ -683,7 +676,7 @@
       <c r="C9" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="2" t="n">
         <v>4.6699999999999997E-5</v>
       </c>
       <c r="E9" t="s">
@@ -696,7 +689,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -706,7 +699,7 @@
       <c r="C10" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="2" t="n">
         <v>1.74E-3</v>
       </c>
       <c r="E10" t="s">
@@ -719,7 +712,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -729,7 +722,7 @@
       <c r="C11" t="s">
         <v>17</v>
       </c>
-      <c r="D11">
+      <c r="D11" t="n">
         <v>0.25</v>
       </c>
       <c r="E11" t="s">
@@ -742,7 +735,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -752,7 +745,7 @@
       <c r="C12" t="s">
         <v>20</v>
       </c>
-      <c r="D12">
+      <c r="D12" t="n">
         <v>0.60899999999999999</v>
       </c>
       <c r="E12" t="s">
@@ -765,7 +758,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" ht="28.5" customHeight="1">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -775,7 +768,7 @@
       <c r="C13" t="s">
         <v>23</v>
       </c>
-      <c r="D13">
+      <c r="D13" t="n">
         <v>4.2599999999999999E-2</v>
       </c>
       <c r="E13" t="s">
@@ -788,7 +781,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -798,7 +791,7 @@
       <c r="C14" t="s">
         <v>9</v>
       </c>
-      <c r="D14">
+      <c r="D14" t="n">
         <v>1.07</v>
       </c>
       <c r="E14" t="s">
@@ -811,7 +804,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" ht="28.5" customHeight="1">
       <c r="A15" t="s">
         <v>32</v>
       </c>
@@ -821,7 +814,7 @@
       <c r="C15" t="s">
         <v>13</v>
       </c>
-      <c r="D15">
+      <c r="D15" t="n">
         <v>1.4499999999999999E-3</v>
       </c>
       <c r="E15" t="s">
@@ -834,7 +827,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:7" s="3" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" ht="28.5" customHeight="1">
       <c r="A16" s="3" t="s">
         <v>32</v>
       </c>
@@ -844,20 +837,20 @@
       <c r="C16" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D16" s="3">
+      <c r="D16" s="3" t="n">
         <v>0.114</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F16" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="G16" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:7" s="3" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" ht="28.5" customHeight="1">
       <c r="A17" s="3" t="s">
         <v>32</v>
       </c>
@@ -867,20 +860,20 @@
       <c r="C17" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D17" s="3">
+      <c r="D17" s="3" t="n">
         <v>2.7E-2</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F17" s="4" t="s">
+      <c r="F17" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G17" s="4" t="s">
+      <c r="G17" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="18" spans="1:7" s="3" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" ht="28.5" customHeight="1">
       <c r="A18" s="3" t="s">
         <v>32</v>
       </c>
@@ -890,20 +883,20 @@
       <c r="C18" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D18" s="3">
+      <c r="D18" s="3" t="n">
         <v>7.1379999999999999E-2</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F18" s="4" t="s">
+      <c r="F18" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G18" s="4" t="s">
+      <c r="G18" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="19" spans="1:7" s="3" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" ht="28.5" customHeight="1">
       <c r="A19" s="3" t="s">
         <v>32</v>
       </c>
@@ -913,20 +906,20 @@
       <c r="C19" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D19" s="3">
+      <c r="D19" s="3" t="n">
         <v>2.7E-2</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F19" s="4" t="s">
+      <c r="F19" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G19" s="4" t="s">
+      <c r="G19" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="20" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="20">
       <c r="A20" s="3" t="s">
         <v>40</v>
       </c>
@@ -936,20 +929,20 @@
       <c r="C20" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D20" s="3">
+      <c r="D20" s="3" t="n">
         <v>8.1000000000000003E-2</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F20" s="4" t="s">
+      <c r="F20" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="G20" s="4" t="s">
+      <c r="G20" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="21">
       <c r="A21" s="3" t="s">
         <v>40</v>
       </c>
@@ -959,20 +952,20 @@
       <c r="C21" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D21" s="5">
+      <c r="D21" s="2" t="n">
         <v>3.1E-4</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F21" s="4" t="s">
+      <c r="F21" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="G21" s="4" t="s">
+      <c r="G21" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="22">
       <c r="A22" s="3" t="s">
         <v>40</v>
       </c>
@@ -982,20 +975,20 @@
       <c r="C22" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D22" s="3">
+      <c r="D22" s="3" t="n">
         <v>1.6999999999999999E-3</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="F22" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="G22" s="4" t="s">
+      <c r="G22" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="23">
       <c r="A23" s="3" t="s">
         <v>40</v>
       </c>
@@ -1005,17 +998,17 @@
       <c r="C23" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D23" s="3">
+      <c r="D23" s="3" t="n">
         <v>2.7E-2</v>
       </c>
-      <c r="F23" s="4" t="s">
+      <c r="F23" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="G23" s="4" t="s">
+      <c r="G23" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="24" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="24">
       <c r="A24" s="3" t="s">
         <v>40</v>
       </c>
@@ -1025,20 +1018,20 @@
       <c r="C24" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D24" s="3">
+      <c r="D24" s="3" t="n">
         <v>7.1379999999999999E-2</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F24" s="4" t="s">
+      <c r="F24" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="G24" s="4" t="s">
+      <c r="G24" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="25" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="25">
       <c r="A25" s="3" t="s">
         <v>40</v>
       </c>
@@ -1048,20 +1041,20 @@
       <c r="C25" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D25" s="3">
+      <c r="D25" s="3" t="n">
         <v>2.7E-2</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F25" s="4" t="s">
+      <c r="F25" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="G25" s="4" t="s">
+      <c r="G25" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="26" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="26">
       <c r="A26" s="3" t="s">
         <v>42</v>
       </c>
@@ -1071,20 +1064,20 @@
       <c r="C26" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D26" s="3">
+      <c r="D26" s="3" t="n">
         <v>1.07</v>
       </c>
       <c r="E26" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F26" s="4" t="s">
+      <c r="F26" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="G26" s="4" t="s">
+      <c r="G26" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="27" spans="1:7" s="3" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" ht="28.5" customHeight="1">
       <c r="A27" s="3" t="s">
         <v>42</v>
       </c>
@@ -1094,20 +1087,20 @@
       <c r="C27" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D27" s="3">
+      <c r="D27" s="3" t="n">
         <v>5.8E-5</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F27" s="4" t="s">
+      <c r="F27" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="G27" s="4" t="s">
+      <c r="G27" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="28" spans="1:7" s="3" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" ht="28.5" customHeight="1">
       <c r="A28" s="3" t="s">
         <v>42</v>
       </c>
@@ -1117,20 +1110,20 @@
       <c r="C28" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D28" s="3">
+      <c r="D28" s="3" t="n">
         <v>1.8600000000000001E-3</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="F28" s="4" t="s">
+      <c r="F28" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="G28" s="4" t="s">
+      <c r="G28" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29">
       <c r="A29" t="s">
         <v>42</v>
       </c>
@@ -1140,7 +1133,7 @@
       <c r="C29" t="s">
         <v>17</v>
       </c>
-      <c r="D29">
+      <c r="D29" t="n">
         <v>0.48</v>
       </c>
       <c r="E29" t="s">
@@ -1153,7 +1146,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30">
       <c r="A30" t="s">
         <v>42</v>
       </c>
@@ -1163,7 +1156,7 @@
       <c r="C30" t="s">
         <v>20</v>
       </c>
-      <c r="D30">
+      <c r="D30" t="n">
         <v>1.2999999999999999E-2</v>
       </c>
       <c r="E30" t="s">
@@ -1176,7 +1169,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="31">
       <c r="A31" t="s">
         <v>42</v>
       </c>
@@ -1186,7 +1179,7 @@
       <c r="C31" t="s">
         <v>23</v>
       </c>
-      <c r="D31">
+      <c r="D31" t="n">
         <v>0.48</v>
       </c>
       <c r="E31" t="s">
@@ -1197,7 +1190,7 @@
       </c>
       <c r="G31" s="1"/>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="32">
       <c r="A32" t="s">
         <v>50</v>
       </c>
@@ -1207,7 +1200,7 @@
       <c r="C32" t="s">
         <v>9</v>
       </c>
-      <c r="D32">
+      <c r="D32" t="n">
         <v>1.07</v>
       </c>
       <c r="E32" t="s">
@@ -1220,7 +1213,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="33">
       <c r="A33" t="s">
         <v>50</v>
       </c>
@@ -1230,7 +1223,7 @@
       <c r="C33" t="s">
         <v>13</v>
       </c>
-      <c r="D33">
+      <c r="D33" t="n">
         <v>1.34E-3</v>
       </c>
       <c r="E33" t="s">
@@ -1243,7 +1236,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="34">
       <c r="A34" t="s">
         <v>50</v>
       </c>
@@ -1253,7 +1246,7 @@
       <c r="C34" t="s">
         <v>15</v>
       </c>
-      <c r="D34">
+      <c r="D34" t="n">
         <v>1.2840000000000001E-2</v>
       </c>
       <c r="E34" t="s">
@@ -1266,7 +1259,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="35">
       <c r="A35" t="s">
         <v>50</v>
       </c>
@@ -1276,7 +1269,7 @@
       <c r="C35" t="s">
         <v>17</v>
       </c>
-      <c r="D35">
+      <c r="D35" t="n">
         <v>0.28000000000000003</v>
       </c>
       <c r="E35" t="s">
@@ -1289,7 +1282,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="36">
       <c r="A36" t="s">
         <v>50</v>
       </c>
@@ -1299,7 +1292,7 @@
       <c r="C36" t="s">
         <v>20</v>
       </c>
-      <c r="D36">
+      <c r="D36" t="n">
         <v>1</v>
       </c>
       <c r="E36" t="s">
@@ -1312,7 +1305,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="37">
       <c r="A37" t="s">
         <v>50</v>
       </c>
@@ -1322,7 +1315,7 @@
       <c r="C37" t="s">
         <v>23</v>
       </c>
-      <c r="D37">
+      <c r="D37" t="n">
         <v>0.28000000000000003</v>
       </c>
       <c r="E37" t="s">
@@ -1335,7 +1328,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="38">
       <c r="A38" t="s">
         <v>57</v>
       </c>
@@ -1345,7 +1338,7 @@
       <c r="C38" t="s">
         <v>9</v>
       </c>
-      <c r="D38">
+      <c r="D38" t="n">
         <v>1.07</v>
       </c>
       <c r="E38" t="s">
@@ -1358,7 +1351,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="39">
       <c r="A39" t="s">
         <v>57</v>
       </c>
@@ -1368,7 +1361,7 @@
       <c r="C39" t="s">
         <v>13</v>
       </c>
-      <c r="D39">
+      <c r="D39" t="n">
         <v>1.27E-4</v>
       </c>
       <c r="E39" t="s">
@@ -1381,7 +1374,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="40">
       <c r="A40" t="s">
         <v>57</v>
       </c>
@@ -1391,7 +1384,7 @@
       <c r="C40" t="s">
         <v>15</v>
       </c>
-      <c r="D40">
+      <c r="D40" t="n">
         <v>9.5999999999999992E-3</v>
       </c>
       <c r="E40" t="s">
@@ -1404,7 +1397,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="41">
       <c r="A41" t="s">
         <v>57</v>
       </c>
@@ -1414,7 +1407,7 @@
       <c r="C41" t="s">
         <v>17</v>
       </c>
-      <c r="D41">
+      <c r="D41" t="n">
         <v>0.86599999999999999</v>
       </c>
       <c r="E41" t="s">
@@ -1427,7 +1420,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="42">
       <c r="A42" t="s">
         <v>57</v>
       </c>
@@ -1437,7 +1430,7 @@
       <c r="C42" t="s">
         <v>20</v>
       </c>
-      <c r="D42">
+      <c r="D42" t="n">
         <v>1E-3</v>
       </c>
       <c r="E42" t="s">
@@ -1450,7 +1443,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="43">
       <c r="A43" t="s">
         <v>57</v>
       </c>
@@ -1460,7 +1453,7 @@
       <c r="C43" t="s">
         <v>23</v>
       </c>
-      <c r="D43">
+      <c r="D43" t="n">
         <v>0.223</v>
       </c>
       <c r="E43" t="s">
@@ -1470,7 +1463,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="44">
       <c r="A44" t="s">
         <v>66</v>
       </c>
@@ -1480,7 +1473,7 @@
       <c r="C44" t="s">
         <v>9</v>
       </c>
-      <c r="D44">
+      <c r="D44" t="n">
         <v>1.07</v>
       </c>
       <c r="E44" t="s">
@@ -1493,7 +1486,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="45">
       <c r="A45" t="s">
         <v>66</v>
       </c>
@@ -1503,7 +1496,7 @@
       <c r="C45" t="s">
         <v>13</v>
       </c>
-      <c r="D45">
+      <c r="D45" t="n">
         <v>1.8E-5</v>
       </c>
       <c r="E45" t="s">
@@ -1516,7 +1509,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="46">
       <c r="A46" t="s">
         <v>66</v>
       </c>
@@ -1526,7 +1519,7 @@
       <c r="C46" t="s">
         <v>15</v>
       </c>
-      <c r="D46">
+      <c r="D46" t="n">
         <v>5.5830000000000003E-3</v>
       </c>
       <c r="E46" t="s">
@@ -1539,7 +1532,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="47">
       <c r="A47" t="s">
         <v>66</v>
       </c>
@@ -1549,7 +1542,7 @@
       <c r="C47" t="s">
         <v>17</v>
       </c>
-      <c r="D47">
+      <c r="D47" t="n">
         <v>0.86599999999999999</v>
       </c>
       <c r="E47" t="s">
@@ -1562,7 +1555,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="48">
       <c r="A48" t="s">
         <v>66</v>
       </c>
@@ -1572,7 +1565,7 @@
       <c r="C48" t="s">
         <v>20</v>
       </c>
-      <c r="D48">
+      <c r="D48" t="n">
         <v>1E-3</v>
       </c>
       <c r="E48" t="s">
@@ -1585,7 +1578,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="49">
       <c r="A49" t="s">
         <v>66</v>
       </c>
@@ -1595,7 +1588,7 @@
       <c r="C49" t="s">
         <v>23</v>
       </c>
-      <c r="D49">
+      <c r="D49" t="n">
         <v>0.223</v>
       </c>
       <c r="E49" t="s">

</xml_diff>